<commit_message>
Support per-payload curl timeouts with three-second defaults
</commit_message>
<xml_diff>
--- a/samples/config.xlsx
+++ b/samples/config.xlsx
@@ -11,13 +11,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Settings!$A$1:$B$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">PayloadTypes!$A$1:$C$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">PayloadTypes!$A$1:$E$61</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="28">
   <si>
     <t>key</t>
   </si>
@@ -46,13 +46,10 @@
     <t>connectTimeoutSeconds</t>
   </si>
   <si>
-    <t>10</t>
+    <t>3</t>
   </si>
   <si>
     <t>requestTimeoutSeconds</t>
-  </si>
-  <si>
-    <t>60</t>
   </si>
   <si>
     <t>outputDirectory</t>
@@ -224,15 +221,15 @@
         <v>10</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>12</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -243,687 +240,695 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="24.0" customWidth="true"/>
-    <col min="2" max="2" width="24.0" customWidth="true"/>
-    <col min="3" max="3" width="24.0" customWidth="true"/>
+    <col min="1" max="1" width="26.0" customWidth="true"/>
+    <col min="2" max="2" width="26.0" customWidth="true"/>
+    <col min="3" max="3" width="26.0" customWidth="true"/>
+    <col min="4" max="4" width="26.0" customWidth="true"/>
+    <col min="5" max="5" width="26.0" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1" ht="24.0" customHeight="true">
       <c r="A1" t="s" s="2">
+        <v>13</v>
+      </c>
+      <c r="B1" t="s" s="2">
         <v>14</v>
       </c>
-      <c r="B1" t="s" s="2">
+      <c r="C1" t="s" s="2">
         <v>15</v>
       </c>
-      <c r="C1" t="s" s="2">
-        <v>16</v>
+      <c r="D1" t="s" s="2">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s" s="2">
+        <v>10</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C52" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C53" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C54" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C56" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C57" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C58" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C60" t="s" s="0">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C61" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C61"/>
+  <autoFilter ref="A1:E61"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Support configurable extra curl arguments and document usage
</commit_message>
<xml_diff>
--- a/samples/config.xlsx
+++ b/samples/config.xlsx
@@ -10,14 +10,14 @@
     <sheet name="PayloadTypes" r:id="rId4" sheetId="2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Settings!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="true">Settings!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="true">PayloadTypes!$A$1:$E$61</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="199" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="30">
   <si>
     <t>key</t>
   </si>
@@ -56,6 +56,12 @@
   </si>
   <si>
     <t>results</t>
+  </si>
+  <si>
+    <t>curlArguments</t>
+  </si>
+  <si>
+    <t>[]</t>
   </si>
   <si>
     <t>contentType</t>
@@ -169,7 +175,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="30.0" customWidth="true"/>
@@ -232,8 +238,16 @@
         <v>12</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B7"/>
+  <autoFilter ref="A1:B8"/>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
@@ -252,13 +266,13 @@
   <sheetData>
     <row r="1" ht="24.0" customHeight="true">
       <c r="A1" t="s" s="2">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B1" t="s" s="2">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C1" t="s" s="2">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D1" t="s" s="2">
         <v>8</v>
@@ -269,662 +283,662 @@
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C14" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C15" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C17" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C19" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C27" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C28" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C29" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C30" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C31" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C32" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C33" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C34" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C35" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C36" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C37" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C38" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C39" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C41" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C42" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C43" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C44" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C45" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s" s="0">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C46" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C47" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C48" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C49" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C50" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C51" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C52" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C53" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C54" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C55" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C56" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C57" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C58" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C59" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C60" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="0">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C61" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>